<commit_message>
feat: consolidate source table config
</commit_message>
<xml_diff>
--- a/conformance/fixtures/001-bracket-substitution/template.xlsx
+++ b/conformance/fixtures/001-bracket-substitution/template.xlsx
@@ -26,7 +26,7 @@
     <t>Data</t>
   </si>
   <si>
-    <t>header_row</t>
+    <t>source_table</t>
   </si>
   <si>
     <t>1</t>
@@ -455,7 +455,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -476,6 +476,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>